<commit_message>
Update history.xlsx with new workshop opening data
Source data for the timeline (rc-app/history.html). The rendered
slide itself needs regenerating (python convert.py in pages/rc-app/)
once we get to page 20 (СТРУКТУРА block) in the new plan.
</commit_message>
<xml_diff>
--- a/pages/rc-app/history.xlsx
+++ b/pages/rc-app/history.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\UU\UCampus\RC_Review\pages\rc-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5B98EF-07F4-445B-A2D5-BDB7B455A333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0055627-5DE4-4DBB-875C-8EEB57508EED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-2750" windowWidth="38620" windowHeight="21100" xr2:uid="{54A213B2-63FF-44EF-85DB-CE274DB8A596}"/>
+    <workbookView xWindow="57480" yWindow="8610" windowWidth="38640" windowHeight="21120" xr2:uid="{54A213B2-63FF-44EF-85DB-CE274DB8A596}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="28">
   <si>
     <t>РЦ</t>
   </si>
@@ -97,6 +97,18 @@
   </si>
   <si>
     <t>ПРОКАТ АНО МШК</t>
+  </si>
+  <si>
+    <t>МАСТЕРСКАЯ ВЯЗАНИЯ</t>
+  </si>
+  <si>
+    <t>КРАСИЛЬНАЯ МАСТЕРСКАЯ</t>
+  </si>
+  <si>
+    <t>ОБРАБОТКА МЕТАЛЛА</t>
+  </si>
+  <si>
+    <t>КЕРАМИКА ОГНЯ</t>
   </si>
 </sst>
 </file>
@@ -467,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835D9306-4152-4C80-BC0E-FC58626EA9EA}">
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.54296875" customWidth="1"/>
@@ -688,10 +700,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>18</v>
@@ -702,41 +714,73 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
-        <v>2030</v>
+        <v>2028</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="A18" s="2">
+        <v>2029</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="A19" s="2">
+        <v>2030</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="A20" s="2">
+        <v>2031</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="A21" s="2">
+        <v>2032</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="2"/>
@@ -858,6 +902,18 @@
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
     </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Page 21 timeline: new workshop names from history.xlsx, no-store data fetch
history.xlsx renames Фотостудия Артплей -> Фотостудия, Тёмная комната
-> Малый даркрум, Шелкография -> Ручная печать and adds Большой даркрум
(2014); history.json regenerated with the same code convert.py uses,
without re-extracting org-chart photos.

The embedded apps fetched their JSON through the browser cache, so the
timeline kept showing the old names after the update; both now fetch
with cache: "no-store".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pages/rc-app/history.xlsx
+++ b/pages/rc-app/history.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\UU\UCampus\RC_Review\pages\rc-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0055627-5DE4-4DBB-875C-8EEB57508EED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1511F9FA-8F38-4A49-A815-9B183C8C9953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8610" windowWidth="38640" windowHeight="21120" xr2:uid="{54A213B2-63FF-44EF-85DB-CE274DB8A596}"/>
+    <workbookView xWindow="38290" yWindow="2210" windowWidth="38620" windowHeight="21100" xr2:uid="{54A213B2-63FF-44EF-85DB-CE274DB8A596}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="29">
   <si>
     <t>РЦ</t>
   </si>
@@ -45,15 +45,6 @@
     <t>3D МАСТЕРСКАЯ</t>
   </si>
   <si>
-    <t>ФОТОСТУДИЯ АРТПЛЕЙ</t>
-  </si>
-  <si>
-    <t>ТЕМНАЯ КОМНАТА</t>
-  </si>
-  <si>
-    <t>ШЕЛКОГРАФИЯ</t>
-  </si>
-  <si>
     <t>КЕРАМИКА</t>
   </si>
   <si>
@@ -109,6 +100,18 @@
   </si>
   <si>
     <t>КЕРАМИКА ОГНЯ</t>
+  </si>
+  <si>
+    <t>МАЛЫЙ ДАРКРУМ</t>
+  </si>
+  <si>
+    <t>ФОТОСТУДИЯ</t>
+  </si>
+  <si>
+    <t>БОЛЬШОЙ ДАРКРУМ</t>
+  </si>
+  <si>
+    <t>РУЧНАЯ ПЕЧАТЬ</t>
   </si>
 </sst>
 </file>
@@ -479,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835D9306-4152-4C80-BC0E-FC58626EA9EA}">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.54296875" customWidth="1"/>
@@ -496,7 +499,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -510,7 +513,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>4</v>
@@ -524,7 +527,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>4</v>
@@ -535,10 +538,10 @@
         <v>2008</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>4</v>
@@ -549,10 +552,10 @@
         <v>2009</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>4</v>
@@ -563,10 +566,10 @@
         <v>2011</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>4</v>
@@ -577,10 +580,10 @@
         <v>2012</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>4</v>
@@ -591,10 +594,10 @@
         <v>2012</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>4</v>
@@ -602,13 +605,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>4</v>
@@ -616,13 +619,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>4</v>
@@ -633,10 +636,10 @@
         <v>2018</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>4</v>
@@ -644,13 +647,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>4</v>
@@ -658,13 +661,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>4</v>
@@ -672,13 +675,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>4</v>
@@ -689,10 +692,10 @@
         <v>2026</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>4</v>
@@ -700,93 +703,101 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
+        <v>2031</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
         <v>2032</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="B22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2"/>
@@ -914,6 +925,12 @@
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
     </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>